<commit_message>
Record Zenodo DOI in manuscript metadata
</commit_message>
<xml_diff>
--- a/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
+++ b/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
@@ -794,18 +794,6 @@
       <c r="L2" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -852,18 +840,6 @@
       <c r="L3" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -910,18 +886,6 @@
       <c r="L4" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -968,18 +932,6 @@
       <c r="L5" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1026,18 +978,6 @@
       <c r="L6" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1084,18 +1024,6 @@
       <c r="L7" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1142,18 +1070,6 @@
       <c r="L8" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1200,18 +1116,6 @@
       <c r="L9" t="n">
         <v>0.2061855670103092</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1234,10 +1138,6 @@
           <t>selected by original-training internal validation; original held-out test evaluated once</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>0.6348039215686275</v>
       </c>
@@ -1262,14 +1162,6 @@
       <c r="P10" t="n">
         <v>34</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1277,17 +1169,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>signal_plus_ssl64_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>0.6559714795008913</v>
       </c>
@@ -1326,10 +1212,6 @@
       <c r="T11" t="n">
         <v>1.025974025974026</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1337,17 +1219,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca5_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>0.6285650623885918</v>
       </c>
@@ -1389,9 +1265,6 @@
       <c r="U12" t="n">
         <v>0.8400092079149173</v>
       </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1399,17 +1272,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca5_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>0.6278966131907309</v>
       </c>
@@ -1451,9 +1318,6 @@
       <c r="U13" t="n">
         <v>0.8400092079149173</v>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1461,17 +1325,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca10_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>0.6212121212121212</v>
       </c>
@@ -1513,9 +1371,6 @@
       <c r="U14" t="n">
         <v>0.9567100820987596</v>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1523,17 +1378,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca10_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>0.6194295900178253</v>
       </c>
@@ -1575,9 +1424,6 @@
       <c r="U15" t="n">
         <v>0.9567100820987596</v>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1585,17 +1431,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca20_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
         <v>0.6535204991087344</v>
       </c>
@@ -1637,9 +1477,6 @@
       <c r="U16" t="n">
         <v>0.9953479552477952</v>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1647,17 +1484,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca20_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>0.6548573975044564</v>
       </c>
@@ -1699,9 +1530,6 @@
       <c r="U17" t="n">
         <v>0.9953479552477952</v>
       </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1709,17 +1537,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>0.6303475935828877</v>
       </c>
@@ -1744,11 +1566,6 @@
       <c r="P18" t="n">
         <v>34</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>neonatal_risk</t>
@@ -1769,17 +1586,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
         <v>0.6559714795008913</v>
       </c>
@@ -1804,11 +1615,6 @@
       <c r="P19" t="n">
         <v>34</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>neonatal_risk</t>
@@ -1829,17 +1635,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>0.6397812713602188</v>
       </c>
@@ -1864,11 +1664,6 @@
       <c r="P20" t="n">
         <v>33</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_15</t>
@@ -1889,17 +1684,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>0.6744133059922534</v>
       </c>
@@ -1924,11 +1713,6 @@
       <c r="P21" t="n">
         <v>33</v>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_15</t>
@@ -1949,17 +1733,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>0.7808807733619764</v>
       </c>
@@ -1984,11 +1762,6 @@
       <c r="P22" t="n">
         <v>19</v>
       </c>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_10</t>
@@ -2009,17 +1782,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
         <v>0.8005728607232366</v>
       </c>
@@ -2044,11 +1811,6 @@
       <c r="P23" t="n">
         <v>19</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_10</t>
@@ -2069,17 +1831,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>0.8181015452538631</v>
       </c>
@@ -2104,11 +1860,6 @@
       <c r="P24" t="n">
         <v>15</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_05</t>
@@ -2129,17 +1880,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>0.8631346578366446</v>
       </c>
@@ -2164,11 +1909,6 @@
       <c r="P25" t="n">
         <v>15</v>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_05</t>
@@ -2939,7 +2679,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Partially reported</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2949,7 +2689,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pipeline scripts are named; public code archive is required before submission.</t>
+          <t>Pipeline scripts are named and the versioned repository archive is available at https://doi.org/10.5281/zenodo.20364142.</t>
         </is>
       </c>
     </row>
@@ -3236,7 +2976,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Partially reported</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -3246,7 +2986,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Local scripts are identified; GitHub/Zenodo archive should be finalized before submission.</t>
+          <t>Local scripts are identified; the GitHub repository and versioned Zenodo archive are reported in Code availability.</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3138,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Partially reported</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3408,7 +3148,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Architecture, feature dimensions and logistic models are described; implementation scripts are included and should be archived publicly.</t>
+          <t>Architecture, feature dimensions and logistic models are described; implementation scripts are included in the GitHub repository and versioned Zenodo archive.</t>
         </is>
       </c>
     </row>
@@ -3719,10 +3459,6 @@
           <t>Open intrapartum FHR and uterine contraction signals with clinical metadata.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3749,10 +3485,6 @@
           <t>Record-level split to avoid window leakage.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3779,10 +3511,6 @@
           <t>Held-out record-level test set for manuscript metrics.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3801,16 +3529,11 @@
       <c r="D5" t="n">
         <v>2604</v>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Used for embedding transport and phenotype assignment, not external outcome validation.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3823,9 +3546,6 @@
           <t>primary raw signal cohort</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>552 intrapartum CTG records with FHR/UC signals and clinical metadata</t>
@@ -3863,9 +3583,6 @@
           <t>feature-level baseline</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>2126 CTG feature rows; no raw signal</t>
@@ -3903,9 +3620,6 @@
           <t>multi-source external/harmonized validation</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Includes CTU-UHB derived files and other sources; SPAM subset notes DUA requirement</t>
@@ -3943,9 +3657,6 @@
           <t>optional expert annotation layer</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Useful for clinically interpretable event annotation if files are accessible</t>
@@ -4143,10 +3854,6 @@
       <c r="D5" t="n">
         <v>-1.383755627705228</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4167,10 +3874,6 @@
       <c r="D6" t="n">
         <v>0.4876152392048818</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4287,10 +3990,6 @@
       <c r="D10" t="n">
         <v>-1.364999581449743</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4311,10 +4010,6 @@
       <c r="D11" t="n">
         <v>0.2456745955547829</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4431,10 +4126,6 @@
       <c r="D15" t="n">
         <v>-1.405010952261644</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4455,10 +4146,6 @@
       <c r="D16" t="n">
         <v>0.4519704801862288</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4575,10 +4262,6 @@
       <c r="D20" t="n">
         <v>-1.367550433996081</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4599,10 +4282,6 @@
       <c r="D21" t="n">
         <v>0.4662218167419979</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4719,10 +4398,6 @@
       <c r="D25" t="n">
         <v>-1.35708270999312</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4743,10 +4418,6 @@
       <c r="D26" t="n">
         <v>-0.7466945871717742</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4863,10 +4534,6 @@
       <c r="D30" t="n">
         <v>-1.377008128000918</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4887,10 +4554,6 @@
       <c r="D31" t="n">
         <v>0.5030790154930093</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5007,10 +4670,6 @@
       <c r="D35" t="n">
         <v>-1.38566366917648</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5031,10 +4690,6 @@
       <c r="D36" t="n">
         <v>0.4739686041976065</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5151,10 +4806,6 @@
       <c r="D40" t="n">
         <v>-1.404498800401032</v>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5175,10 +4826,6 @@
       <c r="D41" t="n">
         <v>0.4731855410006625</v>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6796,14 +6443,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6836,14 +6475,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6876,14 +6507,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6916,14 +6539,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6956,14 +6571,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6996,14 +6603,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7016,11 +6615,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7066,11 +6660,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7116,11 +6705,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7166,11 +6750,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7216,11 +6795,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7266,11 +6840,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7316,11 +6885,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7366,11 +6930,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7416,11 +6975,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7466,11 +7020,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7516,11 +7065,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7566,11 +7110,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7616,11 +7155,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7666,11 +7200,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7716,11 +7245,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7766,11 +7290,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7816,11 +7335,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7866,11 +7380,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7916,11 +7425,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7966,11 +7470,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8016,11 +7515,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8066,11 +7560,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8116,11 +7605,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8166,11 +7650,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8216,11 +7695,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8266,11 +7740,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8316,11 +7785,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8366,11 +7830,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8416,11 +7875,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8466,11 +7920,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8516,11 +7965,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8566,11 +8010,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8616,11 +8055,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8666,11 +8100,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8716,11 +8145,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8766,11 +8190,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8816,11 +8235,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8866,11 +8280,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8916,11 +8325,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8966,11 +8370,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -9016,11 +8415,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -9066,11 +8460,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -9217,9 +8606,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9257,9 +8643,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9297,9 +8680,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9337,9 +8717,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9377,9 +8754,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9417,9 +8791,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9457,9 +8828,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9497,9 +8865,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9537,9 +8902,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9577,9 +8939,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9617,9 +8976,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9657,9 +9013,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9697,9 +9050,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9737,9 +9087,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9777,9 +9124,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9817,9 +9161,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9857,9 +9198,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9897,9 +9235,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9907,14 +9242,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
         <v>-0.0648795817669172</v>
       </c>
@@ -9949,14 +9281,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
         <v>0.0147921687665013</v>
       </c>
@@ -9991,14 +9320,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
         <v>-0.0184311261951511</v>
       </c>
@@ -10033,14 +9359,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
         <v>-0.0589333593912861</v>
       </c>
@@ -10075,14 +9398,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
         <v>0.0073043136483794</v>
       </c>
@@ -10117,14 +9437,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
         <v>-0.0228116638201394</v>
       </c>
@@ -10159,14 +9476,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
         <v>-0.076264787314372</v>
       </c>
@@ -10201,14 +9515,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
         <v>-0.0373073227774457</v>
       </c>
@@ -10243,14 +9554,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
         <v>-0.0042140458305653</v>
       </c>
@@ -10285,14 +9593,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
         <v>-0.07531340156782509</v>
       </c>
@@ -10327,14 +9632,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
         <v>-0.0307590493676202</v>
       </c>
@@ -10369,14 +9671,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
         <v>-0.0075360405434384</v>
       </c>
@@ -10411,14 +9710,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
         <v>-0.042036806038801</v>
       </c>
@@ -10453,14 +9749,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
         <v>-0.0379749437344173</v>
       </c>
@@ -10495,14 +9788,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
         <v>-0.0194426803381451</v>
       </c>
@@ -10537,14 +9827,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
         <v>-0.065986873319355</v>
       </c>
@@ -10579,14 +9866,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
         <v>-0.06580446484173121</v>
       </c>
@@ -10621,14 +9905,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
         <v>-0.0091076400248609</v>
       </c>
@@ -10663,14 +9944,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
         <v>-0.068578312839773</v>
       </c>
@@ -10705,14 +9983,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
         <v>-0.0586554867300895</v>
       </c>
@@ -10747,14 +10022,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
         <v>-0.009151914153215399</v>
       </c>
@@ -10910,12 +10182,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10953,12 +10219,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10996,12 +10256,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11039,12 +10293,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11082,12 +10330,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11125,12 +10367,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11168,12 +10404,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11211,12 +10441,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11254,12 +10478,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11297,12 +10515,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11340,12 +10552,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11383,12 +10589,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11426,12 +10626,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -11469,12 +10663,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11512,12 +10700,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11555,12 +10737,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11598,12 +10774,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -11641,12 +10811,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11684,12 +10848,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11727,12 +10885,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11770,12 +10922,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11813,12 +10959,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11856,12 +10996,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -11899,12 +11033,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11942,12 +11070,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -11985,12 +11107,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12028,12 +11144,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -12071,12 +11181,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -12114,12 +11218,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -12157,12 +11255,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -12200,12 +11292,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -12243,12 +11329,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -12286,12 +11366,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -12329,12 +11403,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -12372,12 +11440,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -12415,12 +11477,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -12458,12 +11514,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -12501,12 +11551,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -12544,12 +11588,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -12587,12 +11625,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -12630,12 +11662,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -12673,12 +11699,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -12716,12 +11736,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -12759,12 +11773,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -12802,12 +11810,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -12845,12 +11847,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -12888,12 +11884,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -12931,12 +11921,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -12974,12 +11958,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -13017,12 +11995,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -13060,12 +12032,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -13103,12 +12069,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -13146,12 +12106,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -13189,12 +12143,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -13232,12 +12180,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -13275,12 +12217,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -13318,12 +12254,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -13361,12 +12291,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -13404,12 +12328,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -13447,12 +12365,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13490,12 +12402,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -13533,12 +12439,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -13576,12 +12476,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -13589,14 +12483,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="n">
         <v>-0.1318444308036309</v>
       </c>
@@ -13619,10 +12510,6 @@
       <c r="K65" t="n">
         <v>-0.0937097736346811</v>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -13630,14 +12517,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="n">
         <v>0.0557232677293967</v>
       </c>
@@ -13660,10 +12544,6 @@
       <c r="K66" t="n">
         <v>0.2048720908474805</v>
       </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -13671,14 +12551,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="n">
         <v>-0.257289982668784</v>
       </c>
@@ -13701,10 +12578,6 @@
       <c r="K67" t="n">
         <v>-0.200548363096473</v>
       </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -13712,14 +12585,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="n">
         <v>0</v>
       </c>
@@ -13742,10 +12612,6 @@
       <c r="K68" t="n">
         <v>0</v>
       </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -13753,14 +12619,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="n">
         <v>0</v>
       </c>
@@ -13783,10 +12646,6 @@
       <c r="K69" t="n">
         <v>0</v>
       </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -13794,14 +12653,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="n">
         <v>-0.1228478459747595</v>
       </c>
@@ -13824,10 +12680,6 @@
       <c r="K70" t="n">
         <v>-0.08640054322174651</v>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -13835,14 +12687,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="n">
         <v>-0.1545991161794524</v>
       </c>
@@ -13865,10 +12714,6 @@
       <c r="K71" t="n">
         <v>0.010780281140433</v>
       </c>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -13876,14 +12721,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="n">
         <v>-0.2543387552890676</v>
       </c>
@@ -13906,10 +12748,6 @@
       <c r="K72" t="n">
         <v>-0.1899886034675202</v>
       </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -13917,14 +12755,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="n">
         <v>-0.0801266947153704</v>
       </c>
@@ -13947,10 +12782,6 @@
       <c r="K73" t="n">
         <v>-0.0346391372083546</v>
       </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13958,14 +12789,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="n">
         <v>-0.0106908994159864</v>
       </c>
@@ -13988,10 +12816,6 @@
       <c r="K74" t="n">
         <v>0.008865501416036699</v>
       </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13999,14 +12823,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="n">
         <v>-0.1431609937559136</v>
       </c>
@@ -14029,10 +12850,6 @@
       <c r="K75" t="n">
         <v>-0.1022387066800633</v>
       </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -14040,14 +12857,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="n">
         <v>0.3014982787840832</v>
       </c>
@@ -14070,10 +12884,6 @@
       <c r="K76" t="n">
         <v>0.790455034554242</v>
       </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -14081,14 +12891,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="n">
         <v>-0.2548569731671434</v>
       </c>
@@ -14111,10 +12918,6 @@
       <c r="K77" t="n">
         <v>-0.2090451321874967</v>
       </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -14122,14 +12925,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="n">
         <v>0</v>
       </c>
@@ -14152,10 +12952,6 @@
       <c r="K78" t="n">
         <v>0</v>
       </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -14163,14 +12959,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="n">
         <v>0</v>
       </c>
@@ -14193,10 +12986,6 @@
       <c r="K79" t="n">
         <v>0</v>
       </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -14204,14 +12993,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="n">
         <v>-0.1330356732242206</v>
       </c>
@@ -14234,10 +13020,6 @@
       <c r="K80" t="n">
         <v>-0.0936409915753878</v>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -14245,14 +13027,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="n">
         <v>-0.1838779905278295</v>
       </c>
@@ -14275,10 +13054,6 @@
       <c r="K81" t="n">
         <v>0.120403657968083</v>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -14286,14 +13061,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="n">
         <v>-0.2579919342372609</v>
       </c>
@@ -14316,10 +13088,6 @@
       <c r="K82" t="n">
         <v>-0.2037470162722904</v>
       </c>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -14327,14 +13095,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="n">
         <v>-0.2438704686642492</v>
       </c>
@@ -14357,10 +13122,6 @@
       <c r="K83" t="n">
         <v>-0.1658978414100166</v>
       </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -14368,14 +13129,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="n">
         <v>-0.0695113160052367</v>
       </c>
@@ -14398,10 +13156,6 @@
       <c r="K84" t="n">
         <v>-0.02254345416202</v>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -14409,14 +13163,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="n">
         <v>-0.1409702670243439</v>
       </c>
@@ -14439,10 +13190,6 @@
       <c r="K85" t="n">
         <v>-0.09905424499950891</v>
       </c>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -14450,14 +13197,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="n">
         <v>0.3792375740982014</v>
       </c>
@@ -14480,10 +13224,6 @@
       <c r="K86" t="n">
         <v>0.9106272070124882</v>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -14491,14 +13231,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="n">
         <v>-0.2554470612196645</v>
       </c>
@@ -14521,10 +13258,6 @@
       <c r="K87" t="n">
         <v>-0.2052418710887075</v>
       </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -14532,14 +13265,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="n">
         <v>0</v>
       </c>
@@ -14562,10 +13292,6 @@
       <c r="K88" t="n">
         <v>0</v>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -14573,14 +13299,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="n">
         <v>0</v>
       </c>
@@ -14603,10 +13326,6 @@
       <c r="K89" t="n">
         <v>0</v>
       </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -14614,14 +13333,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
         <v>-0.1308294074604928</v>
       </c>
@@ -14644,10 +13360,6 @@
       <c r="K90" t="n">
         <v>-0.0905869942669864</v>
       </c>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -14655,14 +13367,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="n">
         <v>-0.2023866731230674</v>
       </c>
@@ -14685,10 +13394,6 @@
       <c r="K91" t="n">
         <v>0.1059575469471127</v>
       </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -14696,14 +13401,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="n">
         <v>-0.2643711461683697</v>
       </c>
@@ -14726,10 +13428,6 @@
       <c r="K92" t="n">
         <v>-0.2044624524982078</v>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -14737,14 +13435,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
         <v>-0.2317235359105727</v>
       </c>
@@ -14767,10 +13462,6 @@
       <c r="K93" t="n">
         <v>-0.1478529768297257</v>
       </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14778,14 +13469,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="n">
         <v>-0.0526167582417581</v>
       </c>
@@ -14808,27 +13496,13 @@
       <c r="K94" t="n">
         <v>-0.0172324800099395</v>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14847,21 +13521,11 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14880,21 +13544,11 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14913,21 +13567,11 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14946,21 +13590,11 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14979,21 +13613,11 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15012,21 +13636,11 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15045,21 +13659,11 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15073,24 +13677,13 @@
       <c r="N102" t="n">
         <v>0.0995787373220114</v>
       </c>
-      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15109,21 +13702,11 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15142,21 +13725,11 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -15175,21 +13748,11 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15208,21 +13771,11 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15241,21 +13794,11 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15274,21 +13817,11 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15307,21 +13840,11 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15340,21 +13863,11 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15373,21 +13886,11 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15406,21 +13909,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15434,24 +13927,13 @@
       <c r="N113" t="n">
         <v>0.0319763924003066</v>
       </c>
-      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
-      <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15470,21 +13952,11 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15503,21 +13975,11 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -15536,21 +13998,11 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
-      <c r="B117" t="inlineStr"/>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15569,21 +14021,11 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15602,21 +14044,11 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15635,21 +14067,11 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15668,21 +14090,11 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15701,21 +14113,11 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15734,21 +14136,11 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15767,21 +14159,11 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15795,24 +14177,13 @@
       <c r="N124" t="n">
         <v>-0.0264837681579565</v>
       </c>
-      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15831,21 +14202,11 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15864,21 +14225,11 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15951,8 +14302,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15968,8 +14317,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15985,8 +14332,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -16002,8 +14347,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -16019,8 +14362,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16036,8 +14377,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16053,8 +14392,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16070,12 +14407,8 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -16089,8 +14422,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -16104,8 +14435,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -16119,8 +14448,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>

</xml_diff>

<commit_message>
Finalize Methods target package cleanup
</commit_message>
<xml_diff>
--- a/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
+++ b/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
@@ -1987,7 +1987,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identifies self-supervised CTG phenotyping and neonatal risk enrichment in the target intrapartum CTG population.</t>
+          <t>Identifies self-supervised CTG trajectory representation and calibrated neonatal risk enrichment in the target intrapartum CTG population.</t>
         </is>
       </c>
     </row>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Structured Background Methods Results Conclusions abstract added for BMC submission.</t>
+          <t>Structured Background Objectives Methods Results Conclusions abstract aligned with Methods of Information in Medicine positioning.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Objective is evaluation of open-data self-supervised CTG phenotyping for calibrated neonatal risk enrichment.</t>
+          <t>Objective is evaluation of an open-data self-supervised CTG trajectory-representation workflow for calibrated neonatal risk enrichment.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update R1 Zenodo DOI
</commit_message>
<xml_diff>
--- a/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
+++ b/manuscript_overleaf/supplementary_tables/Supplementary_Tables_CTGFHT.xlsx
@@ -540,10 +540,6 @@
           <t>Open intrapartum FHR and uterine contraction signals with clinical metadata.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -570,10 +566,6 @@
           <t>Record-level split to avoid window leakage.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -600,10 +592,6 @@
           <t>Held-out record-level test set for manuscript metrics.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -622,16 +610,11 @@
       <c r="D5" t="n">
         <v>2604</v>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Used for embedding transport and phenotype assignment, not external outcome validation.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -644,9 +627,6 @@
           <t>primary raw signal cohort</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>552 intrapartum CTG records with FHR/UC signals and clinical metadata</t>
@@ -684,9 +664,6 @@
           <t>feature-level baseline</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>2126 CTG feature rows; no raw signal</t>
@@ -724,9 +701,6 @@
           <t>multi-source external/harmonized resource</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Includes CTU-UHB derived files and other sources; SPAM subset notes DUA requirement</t>
@@ -764,9 +738,6 @@
           <t>optional expert annotation layer</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Useful for clinically interpretable event annotation if files are accessible</t>
@@ -1555,7 +1526,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Pipeline scripts are named and the versioned repository archive is available at https://doi.org/10.5281/zenodo.20485068.</t>
+          <t>Pipeline scripts are named and the versioned repository archive is available at https://doi.org/10.5281/zenodo.21242760.</t>
         </is>
       </c>
     </row>
@@ -3395,10 +3366,6 @@
       <c r="D5" t="n">
         <v>-1.383755627705228</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3419,10 +3386,6 @@
       <c r="D6" t="n">
         <v>0.4876152392048818</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3539,10 +3502,6 @@
       <c r="D10" t="n">
         <v>-1.361018968210047</v>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3563,10 +3522,6 @@
       <c r="D11" t="n">
         <v>-0.0414509142196207</v>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3683,10 +3638,6 @@
       <c r="D15" t="n">
         <v>-1.359827394810819</v>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3707,10 +3658,6 @@
       <c r="D16" t="n">
         <v>0.3136181611128629</v>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3827,10 +3774,6 @@
       <c r="D20" t="n">
         <v>-1.367550433996081</v>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3851,10 +3794,6 @@
       <c r="D21" t="n">
         <v>0.4662218167419979</v>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3971,10 +3910,6 @@
       <c r="D25" t="n">
         <v>-1.380104498239844</v>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3995,10 +3930,6 @@
       <c r="D26" t="n">
         <v>1.455541101565448</v>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4115,10 +4046,6 @@
       <c r="D30" t="n">
         <v>-1.377008128000917</v>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4139,10 +4066,6 @@
       <c r="D31" t="n">
         <v>0.5030790154929924</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4259,10 +4182,6 @@
       <c r="D35" t="n">
         <v>-1.426342998940758</v>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4283,10 +4202,6 @@
       <c r="D36" t="n">
         <v>0.5601925824855279</v>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4403,10 +4318,6 @@
       <c r="D40" t="n">
         <v>-1.358793987548642</v>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4427,10 +4338,6 @@
       <c r="D41" t="n">
         <v>0.3447612843466913</v>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H41"/>
@@ -6137,14 +6044,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6177,14 +6076,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6217,14 +6108,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6257,14 +6140,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6297,14 +6172,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6337,14 +6204,6 @@
           <t>feature_family_importance</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6357,11 +6216,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6407,11 +6261,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6457,11 +6306,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6507,11 +6351,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6557,11 +6396,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6607,11 +6441,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6657,11 +6486,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6707,11 +6531,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6757,11 +6576,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6807,11 +6621,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6857,11 +6666,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6907,11 +6711,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -6957,11 +6756,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7007,11 +6801,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7057,11 +6846,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7107,11 +6891,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7157,11 +6936,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7207,11 +6981,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7257,11 +7026,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7307,11 +7071,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7357,11 +7116,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7407,11 +7161,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7457,11 +7206,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7507,11 +7251,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7557,11 +7296,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7607,11 +7341,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7657,11 +7386,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7707,11 +7431,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7757,11 +7476,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7807,11 +7521,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7857,11 +7566,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7907,11 +7611,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -7957,11 +7656,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8007,11 +7701,6 @@
           <t>clinical_signal</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8057,11 +7746,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8107,11 +7791,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8157,11 +7836,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8207,11 +7881,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8257,11 +7926,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8307,11 +7971,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8357,11 +8016,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8407,11 +8061,6 @@
           <t>ssl_embedding</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>top_feature_importance</t>
@@ -8573,9 +8222,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8613,9 +8259,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8653,9 +8296,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8693,9 +8333,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8733,9 +8370,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8773,9 +8407,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8813,9 +8444,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8853,9 +8481,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8893,9 +8518,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8933,9 +8555,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8973,9 +8592,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9013,9 +8629,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9053,9 +8666,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9093,9 +8703,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9133,9 +8740,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9173,9 +8777,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9213,9 +8814,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9253,9 +8851,6 @@
           <t>scenario_metrics</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9263,14 +8858,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
         <v>-0.1152801925126565</v>
       </c>
@@ -9305,14 +8897,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
         <v>-0.0527365042591424</v>
       </c>
@@ -9347,14 +8936,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
         <v>-0.0066880104926575</v>
       </c>
@@ -9389,14 +8975,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
         <v>-0.1011829851497608</v>
       </c>
@@ -9431,14 +9014,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
         <v>-0.0353813521827991</v>
       </c>
@@ -9473,14 +9053,11 @@
           <t>full_features</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
         <v>-0.0128540197111931</v>
       </c>
@@ -9515,14 +9092,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="n">
         <v>-0.1206789120391428</v>
       </c>
@@ -9557,14 +9131,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="n">
         <v>-0.07015807799443639</v>
       </c>
@@ -9599,14 +9170,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="n">
         <v>0.0025525147113689</v>
       </c>
@@ -9641,14 +9209,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
         <v>-0.1200222082547664</v>
       </c>
@@ -9683,14 +9248,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="n">
         <v>-0.069068605127595</v>
       </c>
@@ -9725,14 +9287,11 @@
           <t>no_missingness_features</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
         <v>-0.0010717499700588</v>
       </c>
@@ -9767,14 +9326,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
         <v>-0.042036806038801</v>
       </c>
@@ -9809,14 +9365,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="n">
         <v>-0.0379749437344173</v>
       </c>
@@ -9851,14 +9404,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="n">
         <v>-0.019442680338145</v>
       </c>
@@ -9893,14 +9443,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
         <v>-0.0706653995909214</v>
       </c>
@@ -9935,14 +9482,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
         <v>-0.031251684027421</v>
       </c>
@@ -9977,14 +9521,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
         <v>-0.0192217858307846</v>
       </c>
@@ -10019,14 +9560,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
         <v>-0.0818210420337276</v>
       </c>
@@ -10061,14 +9599,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
         <v>-0.0525863966100343</v>
       </c>
@@ -10103,14 +9638,11 @@
           <t>no_missingness_features vs full_features</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
         <v>-0.0184962137927309</v>
       </c>
@@ -10284,12 +9816,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10327,12 +9853,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10370,12 +9890,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10413,12 +9927,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10456,12 +9964,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10499,12 +10001,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10542,12 +10038,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10585,12 +10075,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10628,12 +10112,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10671,12 +10149,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10714,12 +10186,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10757,12 +10223,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10800,12 +10260,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10843,12 +10297,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10886,12 +10334,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10929,12 +10371,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10972,12 +10408,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -11015,12 +10445,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11058,12 +10482,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11101,12 +10519,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11144,12 +10556,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -11187,12 +10593,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11230,12 +10630,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -11273,12 +10667,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11316,12 +10704,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -11359,12 +10741,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -11402,12 +10778,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -11445,12 +10815,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -11488,12 +10852,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -11531,12 +10889,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -11574,12 +10926,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -11617,12 +10963,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -11660,12 +11000,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -11703,12 +11037,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -11746,12 +11074,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -11789,12 +11111,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -11832,12 +11148,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -11875,12 +11185,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -11918,12 +11222,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -11961,12 +11259,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -12004,12 +11296,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -12047,12 +11333,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -12090,12 +11370,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -12133,12 +11407,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -12176,12 +11444,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -12219,12 +11481,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
-      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -12262,12 +11518,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -12305,12 +11555,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -12348,12 +11592,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -12391,12 +11629,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -12434,12 +11666,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -12477,12 +11703,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
-      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -12520,12 +11740,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="inlineStr"/>
-      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12563,12 +11777,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12606,12 +11814,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -12649,12 +11851,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -12692,12 +11888,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -12735,12 +11925,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -12778,12 +11962,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -12821,12 +11999,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
-      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -12864,12 +12036,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
-      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -12907,12 +12073,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
-      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -12950,12 +12110,6 @@
           <t>recalibration_metrics</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -12963,14 +12117,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="n">
         <v>-0.1318444308036308</v>
       </c>
@@ -12993,10 +12144,6 @@
       <c r="K65" t="n">
         <v>-0.0937097736346811</v>
       </c>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
-      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -13004,14 +12151,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="n">
         <v>0.0557232677293965</v>
       </c>
@@ -13034,10 +12178,6 @@
       <c r="K66" t="n">
         <v>0.2048720908474801</v>
       </c>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -13045,14 +12185,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="n">
         <v>-0.257289982668784</v>
       </c>
@@ -13075,10 +12212,6 @@
       <c r="K67" t="n">
         <v>-0.200548363096473</v>
       </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
-      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -13086,14 +12219,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="n">
         <v>0</v>
       </c>
@@ -13116,10 +12246,6 @@
       <c r="K68" t="n">
         <v>0</v>
       </c>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -13127,14 +12253,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="n">
         <v>0</v>
       </c>
@@ -13157,10 +12280,6 @@
       <c r="K69" t="n">
         <v>0</v>
       </c>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
-      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -13168,14 +12287,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="n">
         <v>-0.1228478459747595</v>
       </c>
@@ -13198,10 +12314,6 @@
       <c r="K70" t="n">
         <v>-0.08640054322174651</v>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
-      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -13209,14 +12321,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="n">
         <v>-0.1545991161794523</v>
       </c>
@@ -13239,10 +12348,6 @@
       <c r="K71" t="n">
         <v>0.0107802811404331</v>
       </c>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="inlineStr"/>
-      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -13250,14 +12355,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="n">
         <v>-0.2543387552890676</v>
       </c>
@@ -13280,10 +12382,6 @@
       <c r="K72" t="n">
         <v>-0.1899886034675202</v>
       </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -13291,14 +12389,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="n">
         <v>-0.0801266947153704</v>
       </c>
@@ -13321,10 +12416,6 @@
       <c r="K73" t="n">
         <v>-0.0346391372083546</v>
       </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
-      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -13332,14 +12423,11 @@
           <t>signal_features</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="n">
         <v>-0.0106908994159864</v>
       </c>
@@ -13362,10 +12450,6 @@
       <c r="K74" t="n">
         <v>0.008865501416036699</v>
       </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="inlineStr"/>
-      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -13373,14 +12457,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="n">
         <v>-0.1550956613943337</v>
       </c>
@@ -13403,10 +12484,6 @@
       <c r="K75" t="n">
         <v>-0.112415817991853</v>
       </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -13414,14 +12491,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="n">
         <v>0.09645057851047489</v>
       </c>
@@ -13444,10 +12518,6 @@
       <c r="K76" t="n">
         <v>0.6326715796329221</v>
       </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -13455,14 +12525,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="n">
         <v>-0.2550918394956318</v>
       </c>
@@ -13485,10 +12552,6 @@
       <c r="K77" t="n">
         <v>-0.2053277010867896</v>
       </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -13496,14 +12559,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="n">
         <v>0</v>
       </c>
@@ -13526,10 +12586,6 @@
       <c r="K78" t="n">
         <v>0</v>
       </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -13537,14 +12593,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="n">
         <v>0</v>
       </c>
@@ -13567,10 +12620,6 @@
       <c r="K79" t="n">
         <v>0</v>
       </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="inlineStr"/>
-      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -13578,14 +12627,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="n">
         <v>-0.1447159308613191</v>
       </c>
@@ -13608,10 +12654,6 @@
       <c r="K80" t="n">
         <v>-0.1041612441249597</v>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -13619,14 +12661,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="n">
         <v>-0.1522148698684831</v>
       </c>
@@ -13649,10 +12688,6 @@
       <c r="K81" t="n">
         <v>0.1198602690872946</v>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -13660,14 +12695,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="n">
         <v>-0.2560144842035606</v>
       </c>
@@ -13690,10 +12722,6 @@
       <c r="K82" t="n">
         <v>-0.1981653902527518</v>
       </c>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -13701,14 +12729,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="n">
         <v>-0.2113114678778499</v>
       </c>
@@ -13731,10 +12756,6 @@
       <c r="K83" t="n">
         <v>-0.1224665696105316</v>
       </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -13742,14 +12763,11 @@
           <t>signal_plus_ssl</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="n">
         <v>-0.0351296647691335</v>
       </c>
@@ -13772,10 +12790,6 @@
       <c r="K84" t="n">
         <v>-0.0104958884627576</v>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -13783,14 +12797,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="n">
         <v>-0.1516015842808508</v>
       </c>
@@ -13813,10 +12824,6 @@
       <c r="K85" t="n">
         <v>-0.1085244293966012</v>
       </c>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -13824,14 +12831,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="n">
         <v>0.2052593036755091</v>
       </c>
@@ -13854,10 +12858,6 @@
       <c r="K86" t="n">
         <v>0.8224879789502427</v>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="inlineStr"/>
-      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -13865,14 +12865,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="n">
         <v>-0.2588395591215532</v>
       </c>
@@ -13895,10 +12892,6 @@
       <c r="K87" t="n">
         <v>-0.2050293349869115</v>
       </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="inlineStr"/>
-      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -13906,14 +12899,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="n">
         <v>0</v>
       </c>
@@ -13936,10 +12926,6 @@
       <c r="K88" t="n">
         <v>0</v>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -13947,14 +12933,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="n">
         <v>0</v>
       </c>
@@ -13977,10 +12960,6 @@
       <c r="K89" t="n">
         <v>0</v>
       </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
-      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -13988,14 +12967,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>brier</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
         <v>-0.1433699315547658</v>
       </c>
@@ -14018,10 +12994,6 @@
       <c r="K90" t="n">
         <v>-0.1027496160442885</v>
       </c>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
-      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -14029,14 +13001,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>calibration_slope</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="n">
         <v>-0.0975750183394154</v>
       </c>
@@ -14059,10 +13028,6 @@
       <c r="K91" t="n">
         <v>0.2034824196229719</v>
       </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="inlineStr"/>
-      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -14070,14 +13035,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>expected_calibration_error</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="n">
         <v>-0.2629659182147544</v>
       </c>
@@ -14100,10 +13062,6 @@
       <c r="K92" t="n">
         <v>-0.2064733282406018</v>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -14111,14 +13069,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>auprc</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
         <v>-0.2365902845470238</v>
       </c>
@@ -14141,10 +13096,6 @@
       <c r="K93" t="n">
         <v>-0.135142218817246</v>
       </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -14152,14 +13103,11 @@
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>auroc</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="n">
         <v>-0.0606345419847327</v>
       </c>
@@ -14182,27 +13130,13 @@
       <c r="K94" t="n">
         <v>-0.026254777816535</v>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
-      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr"/>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
       <c r="I95" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14221,21 +13155,11 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14254,21 +13178,11 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14287,21 +13201,11 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14320,21 +13224,11 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14353,21 +13247,11 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
       <c r="I100" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14386,21 +13270,11 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr"/>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
       <c r="I101" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14419,21 +13293,11 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
       <c r="I102" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14447,24 +13311,13 @@
       <c r="N102" t="n">
         <v>0.1011685988762308</v>
       </c>
-      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr"/>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
       <c r="I103" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14483,21 +13336,11 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" t="inlineStr"/>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14516,21 +13359,11 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
-      <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
           <t>0.05-0.20</t>
@@ -14549,21 +13382,11 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr"/>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
       <c r="I106" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14582,21 +13405,11 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" t="inlineStr"/>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
       <c r="I107" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14615,21 +13428,11 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" t="inlineStr"/>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
       <c r="I108" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14648,21 +13451,11 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
       <c r="I109" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14681,21 +13474,11 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr"/>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
       <c r="I110" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14714,21 +13497,11 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14747,21 +13520,11 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr"/>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
-      <c r="D112" t="inlineStr"/>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
       <c r="I112" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14780,21 +13543,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
-      <c r="D113" t="inlineStr"/>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14808,24 +13561,13 @@
       <c r="N113" t="n">
         <v>0.0260858359978545</v>
       </c>
-      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr"/>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
-      <c r="D114" t="inlineStr"/>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14844,21 +13586,11 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr"/>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr"/>
-      <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
       <c r="I115" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14877,21 +13609,11 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>0.10-0.30</t>
@@ -14910,21 +13632,11 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" t="inlineStr"/>
-      <c r="B117" t="inlineStr"/>
-      <c r="C117" t="inlineStr"/>
-      <c r="D117" t="inlineStr"/>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
       <c r="I117" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -14943,21 +13655,11 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr"/>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
-      <c r="D118" t="inlineStr"/>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -14976,21 +13678,11 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
-      <c r="D119" t="inlineStr"/>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
       <c r="I119" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15009,21 +13701,11 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr"/>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15042,21 +13724,11 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" t="inlineStr"/>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15075,21 +13747,11 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" t="inlineStr"/>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15108,21 +13770,11 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" t="inlineStr"/>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15141,21 +13793,11 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" t="inlineStr"/>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
       <c r="I124" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15169,24 +13811,13 @@
       <c r="N124" t="n">
         <v>-0.034507701619945</v>
       </c>
-      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15205,21 +13836,11 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" t="inlineStr"/>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
-      <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15238,21 +13859,11 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>decision_curve_summary</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
           <t>0.05-0.50</t>
@@ -15333,8 +13944,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15350,8 +13959,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15367,8 +13974,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15384,8 +13989,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15401,8 +14004,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -15418,8 +14019,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -15435,8 +14034,6 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15452,12 +14049,8 @@
           <t>external_embedding_metrics</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -15471,8 +14064,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -15486,8 +14077,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -15501,8 +14090,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>assigned_ssl_phenotype_counts</t>
@@ -15723,18 +14310,6 @@
       <c r="L2" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -15781,18 +14356,6 @@
       <c r="L3" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15839,18 +14402,6 @@
       <c r="L4" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -15897,18 +14448,6 @@
       <c r="L5" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15955,18 +14494,6 @@
       <c r="L6" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -16013,18 +14540,6 @@
       <c r="L7" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16071,18 +14586,6 @@
       <c r="L8" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -16129,18 +14632,6 @@
       <c r="L9" t="n">
         <v>0.2061855670103093</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -16163,10 +14654,6 @@
           <t>selected by original-training internal validation; original held-out test evaluated once</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>0.6348039215686275</v>
       </c>
@@ -16191,14 +14678,6 @@
       <c r="P10" t="n">
         <v>34</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -16206,17 +14685,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>signal_plus_ssl64_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>0.6167557932263814</v>
       </c>
@@ -16255,10 +14728,6 @@
       <c r="T11" t="n">
         <v>1.025974025974026</v>
       </c>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -16266,17 +14735,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca5_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>0.6285650623885918</v>
       </c>
@@ -16318,9 +14781,6 @@
       <c r="U12" t="n">
         <v>0.8400092079149173</v>
       </c>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -16328,17 +14788,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca5_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>0.6278966131907309</v>
       </c>
@@ -16380,9 +14834,6 @@
       <c r="U13" t="n">
         <v>0.8400092079149173</v>
       </c>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -16390,17 +14841,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca10_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
         <v>0.6212121212121212</v>
       </c>
@@ -16442,9 +14887,6 @@
       <c r="U14" t="n">
         <v>0.9567100820987597</v>
       </c>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -16452,17 +14894,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca10_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>0.6194295900178253</v>
       </c>
@@ -16504,9 +14940,6 @@
       <c r="U15" t="n">
         <v>0.9567100820987597</v>
       </c>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -16514,17 +14947,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca20_plus_signal_phenotype_l2</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
         <v>0.6535204991087344</v>
       </c>
@@ -16566,9 +14993,6 @@
       <c r="U16" t="n">
         <v>0.9953479552477952</v>
       </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16576,17 +15000,11 @@
           <t>dimensionality_regularization</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>signal_plus_ssl_pca20_plus_signal_phenotype_elasticnet</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>0.6548573975044564</v>
       </c>
@@ -16628,9 +15046,6 @@
       <c r="U17" t="n">
         <v>0.9953479552477952</v>
       </c>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -16638,17 +15053,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
         <v>0.6303475935828877</v>
       </c>
@@ -16673,11 +15082,6 @@
       <c r="P18" t="n">
         <v>34</v>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr">
         <is>
           <t>neonatal_risk</t>
@@ -16698,17 +15102,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
         <v>0.6167557932263814</v>
       </c>
@@ -16733,11 +15131,6 @@
       <c r="P19" t="n">
         <v>34</v>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr">
         <is>
           <t>neonatal_risk</t>
@@ -16758,17 +15151,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
         <v>0.6397812713602188</v>
       </c>
@@ -16793,11 +15180,6 @@
       <c r="P20" t="n">
         <v>33</v>
       </c>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_15</t>
@@ -16818,17 +15200,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>0.6744133059922534</v>
       </c>
@@ -16853,11 +15229,6 @@
       <c r="P21" t="n">
         <v>33</v>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_15</t>
@@ -16878,17 +15249,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
         <v>0.7808807733619764</v>
       </c>
@@ -16913,11 +15278,6 @@
       <c r="P22" t="n">
         <v>19</v>
       </c>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_10</t>
@@ -16938,17 +15298,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
         <v>0.8005728607232366</v>
       </c>
@@ -16973,11 +15327,6 @@
       <c r="P23" t="n">
         <v>19</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
       <c r="V23" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_10</t>
@@ -16998,17 +15347,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>signal_features</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
         <v>0.8181015452538631</v>
       </c>
@@ -17033,11 +15376,6 @@
       <c r="P24" t="n">
         <v>15</v>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_05</t>
@@ -17058,17 +15396,11 @@
           <t>outcome_sensitivity</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>signal_plus_ssl_plus_signal_phenotype</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
         <v>0.8631346578366446</v>
       </c>
@@ -17093,11 +15425,6 @@
       <c r="P25" t="n">
         <v>15</v>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
       <c r="V25" t="inlineStr">
         <is>
           <t>cord_ph_lt_7_05</t>

</xml_diff>